<commit_message>
Altura a canal por defecto 4,5 m: primera de la lista del catálogo
- Plantilla: alturas de MT-GOT-80 ordenadas como 4.5;4;5
- JSON regenerado; pruebas del motor sin cambios (144, 0 fallos)
- Al cambiar de modelo, la interfaz vuelve a la primera anchura,
  separación y altura de su lista

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DZJD52KrF7GMG33CxptRSh
</commit_message>
<xml_diff>
--- a/datos/Catalogo_Plantilla_v0.4.xlsx
+++ b/datos/Catalogo_Plantilla_v0.4.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresa" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modelos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfiles" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componentes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cubiertas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Obra local" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Empresa" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Modelos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Perfiles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Componentes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cubiertas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Equipos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Obra local" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Variables" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>4;4.5;5</t>
+          <t>4.5;4;5</t>
         </is>
       </c>
       <c r="G6" s="9" t="n">

</xml_diff>

<commit_message>
Catálogo: ancho y alto de puerta en la hoja Equipos
- Plantilla: columnas «Ancho puerta» y «Alto puerta» (m) antes de
  Precio; la puerta de ejemplo mide 3 × 3 m (origen estimado)
- Importador y catalogo_a_json.py: se pasan a número si vienen como
  texto; validador: puerta sin medidas → aviso (no se dibujará),
  medida no numérica o ≤ 0 → error
- Catálogo con errores provocados: una medida de puerta no válida

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DZJD52KrF7GMG33CxptRSh
</commit_message>
<xml_diff>
--- a/datos/Catalogo_Plantilla_v0.4.xlsx
+++ b/datos/Catalogo_Plantilla_v0.4.xlsx
@@ -3558,7 +3558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3570,8 +3570,10 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3588,6 +3590,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -3636,10 +3639,20 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
+          <t>Ancho puerta</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Alto puerta</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="M4" s="7" t="inlineStr">
         <is>
           <t>Origen</t>
         </is>
@@ -3685,10 +3698,20 @@
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
+          <t>m (puertas)</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>m (puertas)</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
           <t>€</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr"/>
+      <c r="M5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -3718,10 +3741,12 @@
       <c r="G6" s="9" t="inlineStr"/>
       <c r="H6" s="9" t="inlineStr"/>
       <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="n">
+      <c r="J6" s="9" t="n"/>
+      <c r="K6" s="9" t="n"/>
+      <c r="L6" s="9" t="n">
         <v>449</v>
       </c>
-      <c r="K6" s="9" t="inlineStr">
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>tienda</t>
         </is>
@@ -3755,10 +3780,12 @@
       <c r="G7" s="9" t="inlineStr"/>
       <c r="H7" s="9" t="inlineStr"/>
       <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="9" t="n">
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="9" t="n"/>
+      <c r="L7" s="9" t="n">
         <v>593</v>
       </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="M7" s="9" t="inlineStr">
         <is>
           <t>tienda</t>
         </is>
@@ -3786,10 +3813,12 @@
       <c r="G8" s="9" t="inlineStr"/>
       <c r="H8" s="9" t="inlineStr"/>
       <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="n">
+      <c r="J8" s="9" t="n"/>
+      <c r="K8" s="9" t="n"/>
+      <c r="L8" s="9" t="n">
         <v>600</v>
       </c>
-      <c r="K8" s="9" t="inlineStr">
+      <c r="M8" s="9" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -3818,9 +3847,15 @@
       <c r="H9" s="9" t="inlineStr"/>
       <c r="I9" s="9" t="inlineStr"/>
       <c r="J9" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" s="9" t="n">
         <v>420</v>
       </c>
-      <c r="K9" s="9" t="inlineStr">
+      <c r="M9" s="9" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -3852,8 +3887,10 @@
         <v>1</v>
       </c>
       <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr">
+      <c r="J10" s="9" t="n"/>
+      <c r="K10" s="9" t="n"/>
+      <c r="L10" s="9" t="n"/>
+      <c r="M10" s="9" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -3885,8 +3922,10 @@
         <v>1</v>
       </c>
       <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr">
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="9" t="n"/>
+      <c r="M11" s="9" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -3916,19 +3955,62 @@
       <c r="I12" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr">
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="9" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="B6:B53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"motor,cuadro,puerta,ventana"</formula1>
     </dataValidation>
-    <dataValidation sqref="K6:K53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M6:M53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"fabricante,literatura,tienda,estimado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Catálogo: columna «Base del viento declarado» en la hoja Modelos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DZJD52KrF7GMG33CxptRSh
</commit_message>
<xml_diff>
--- a/datos/Catalogo_Plantilla_v0.4.xlsx
+++ b/datos/Catalogo_Plantilla_v0.4.xlsx
@@ -853,7 +853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -876,6 +876,7 @@
     <col width="9" customWidth="1" min="18" max="18"/>
     <col width="40" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -993,6 +994,11 @@
           <t>Origen</t>
         </is>
       </c>
+      <c r="U4" s="7" t="inlineStr">
+        <is>
+          <t>Base del viento declarado</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr"/>
@@ -1083,6 +1089,11 @@
         </is>
       </c>
       <c r="T5" s="8" t="inlineStr"/>
+      <c r="U5" s="8" t="inlineStr">
+        <is>
+          <t>velocidad media / ráfaga / presión kN/m²</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1161,6 +1172,7 @@
           <t>estimado</t>
         </is>
       </c>
+      <c r="U6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1239,11 +1251,15 @@
           <t>estimado</t>
         </is>
       </c>
+      <c r="U7" s="9" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="T6:T48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"fabricante,literatura,tienda,estimado"</formula1>
+    </dataValidation>
+    <dataValidation sqref="U6:U48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"velocidad media,ráfaga,presión kN/m²"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3558,7 +3574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3590,7 +3606,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -3964,47 +3979,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="B6:B53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>